<commit_message>
Updated setting ita_core_news_lg Spacy model
</commit_message>
<xml_diff>
--- a/data/reports/atlas_openaire.xlsx
+++ b/data/reports/atlas_openaire.xlsx
@@ -413,9 +413,376 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>atlas_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>titolo_atlas</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>tipo_entita</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>metodo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>count_title</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>count_desc</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>count_subject</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>https://w3id.org/dh-atlas/1743001065-375169</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Il quaderno di Paolo Bufalini - Edizione digitale</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Paolo Bufalini - Edizione</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>KEYWORD</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>NER+KP</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>https://w3id.org/dh-atlas/1743001065-375169</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Il quaderno di Paolo Bufalini - Edizione digitale</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Paolo Bufalini</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>KEYWORD</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NER+KP</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>https://w3id.org/dh-atlas/1743001065-375169</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Il quaderno di Paolo Bufalini - Edizione digitale</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Edizione digitale</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>KEYWORD</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>NER+KP</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>169</v>
+      </c>
+      <c r="G4" t="n">
+        <v>521</v>
+      </c>
+      <c r="H4" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>https://w3id.org/dh-atlas/1743001065-375169</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Il quaderno di Paolo Bufalini - Edizione digitale</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>quaderno di Paolo</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>KEYWORD</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>NER+KP</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>11</v>
+      </c>
+      <c r="G5" t="n">
+        <v>34</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>https://w3id.org/dh-atlas/1743001065-375169</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Il quaderno di Paolo Bufalini - Edizione digitale</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Bufalini</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>KEYWORD</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>NER+KP</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>123</v>
+      </c>
+      <c r="G6" t="n">
+        <v>173</v>
+      </c>
+      <c r="H6" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>https://w3id.org/dh-atlas/1743001065-375169</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Il quaderno di Paolo Bufalini - Edizione digitale</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Edizione</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>KEYWORD</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NER+KP</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>10851</v>
+      </c>
+      <c r="G7" t="n">
+        <v>16082</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2099</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>https://w3id.org/dh-atlas/1743001065-375169</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Il quaderno di Paolo Bufalini - Edizione digitale</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Paolo</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>KEYWORD</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>NER+KP</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>21124</v>
+      </c>
+      <c r="G8" t="n">
+        <v>32743</v>
+      </c>
+      <c r="H8" t="n">
+        <v>5091</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>https://w3id.org/dh-atlas/1743001065-375169</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Il quaderno di Paolo Bufalini - Edizione digitale</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>digitale</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>KEYWORD</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>NER+KP</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>71832</v>
+      </c>
+      <c r="G9" t="n">
+        <v>166038</v>
+      </c>
+      <c r="H9" t="n">
+        <v>54711</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>https://w3id.org/dh-atlas/1743001065-375169</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Il quaderno di Paolo Bufalini - Edizione digitale</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>quaderno</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>KEYWORD</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>NER+KP</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1227</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1497</v>
+      </c>
+      <c r="H10" t="n">
+        <v>66</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>